<commit_message>
v2.0 final: speed 0x158 (primary), MONITOR RAW only, sensors fixed, service manual, canny.ru database
</commit_message>
<xml_diff>
--- a/Honda_Toyota_CAN_ID_Map.xlsx
+++ b/Honda_Toyota_CAN_ID_Map.xlsx
@@ -8,11 +8,20 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Общая информация" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="P-CAN - F-CAN (500 kbps)" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="B-CAN (125 kbps)" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="M-CAN (500 kbps)" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Неизвестно" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Toyota + Lexus" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mercedes W203 W463 (руль)" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mercedes W204 (шатл)" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mercedes Viano W639 (OBF)" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mercedes S W221 (сиденья)" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="BMW E8x E9x Mini" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mazda 3 CX-5" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Peugeot 508" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ford Focus 3" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Opel Corsa D" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="P-CAN - F-CAN (500 kbps)" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="B-CAN (125 kbps)" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="M-CAN (500 kbps)" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Неизвестно" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Toyota + Lexus" sheetId="15" state="visible" r:id="rId15"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -22,7 +31,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="33">
+  <fonts count="34">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -175,8 +184,11 @@
       <b val="1"/>
       <sz val="10"/>
     </font>
+    <font>
+      <sz val="9"/>
+    </font>
   </fonts>
-  <fills count="13">
+  <fills count="15">
     <fill>
       <patternFill/>
     </fill>
@@ -249,6 +261,18 @@
         <bgColor rgb="00FFEB9C"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="004472C4"/>
+        <bgColor rgb="004472C4"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D9E2F3"/>
+        <bgColor rgb="00D9E2F3"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -268,7 +292,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="59">
+  <cellXfs count="62">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -370,6 +394,11 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="13" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="33" fillId="14" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="33" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -1713,7 +1742,573 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E23"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="9" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="33" customWidth="1" min="3" max="3"/>
+    <col width="36" customWidth="1" min="4" max="4"/>
+    <col width="32" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="59" t="inlineStr">
+        <is>
+          <t>CAN ID</t>
+        </is>
+      </c>
+      <c r="B1" s="59" t="inlineStr">
+        <is>
+          <t>Шина</t>
+        </is>
+      </c>
+      <c r="C1" s="59" t="inlineStr">
+        <is>
+          <t>Байт/Бит</t>
+        </is>
+      </c>
+      <c r="D1" s="59" t="inlineStr">
+        <is>
+          <t>Назначение</t>
+        </is>
+      </c>
+      <c r="E1" s="59" t="inlineStr">
+        <is>
+          <t>Примечание</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="60" t="inlineStr">
+        <is>
+          <t>0x370</t>
+        </is>
+      </c>
+      <c r="B2" s="60" t="inlineStr">
+        <is>
+          <t>SWCAN</t>
+        </is>
+      </c>
+      <c r="C2" s="60" t="inlineStr">
+        <is>
+          <t>byte[1]=0x01/0x00</t>
+        </is>
+      </c>
+      <c r="D2" s="60" t="inlineStr">
+        <is>
+          <t>Ручной тормоз: вкл/выкл</t>
+        </is>
+      </c>
+      <c r="E2" s="60" t="inlineStr">
+        <is>
+          <t>SWCAN 33.3kbps / Corsa D 2011</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="61" t="inlineStr">
+        <is>
+          <t>0x350</t>
+        </is>
+      </c>
+      <c r="B3" s="61" t="inlineStr">
+        <is>
+          <t>SWCAN</t>
+        </is>
+      </c>
+      <c r="C3" s="61" t="inlineStr">
+        <is>
+          <t>byte[0] &amp; 0x08</t>
+        </is>
+      </c>
+      <c r="D3" s="61" t="inlineStr">
+        <is>
+          <t>Задний ход (фонарь)</t>
+        </is>
+      </c>
+      <c r="E3" s="61" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="60" t="inlineStr">
+        <is>
+          <t>0x350</t>
+        </is>
+      </c>
+      <c r="B4" s="60" t="inlineStr">
+        <is>
+          <t>SWCAN</t>
+        </is>
+      </c>
+      <c r="C4" s="60" t="inlineStr">
+        <is>
+          <t>byte[0] &amp; 0x04</t>
+        </is>
+      </c>
+      <c r="D4" s="60" t="inlineStr">
+        <is>
+          <t>Габаритные огни</t>
+        </is>
+      </c>
+      <c r="E4" s="60" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="61" t="inlineStr">
+        <is>
+          <t>0x175</t>
+        </is>
+      </c>
+      <c r="B5" s="61" t="inlineStr">
+        <is>
+          <t>SWCAN</t>
+        </is>
+      </c>
+      <c r="C5" s="61" t="inlineStr">
+        <is>
+          <t>byte[5:7]</t>
+        </is>
+      </c>
+      <c r="D5" s="61" t="inlineStr">
+        <is>
+          <t>Кнопки мультимедиа на руле</t>
+        </is>
+      </c>
+      <c r="E5" s="61" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="60" t="inlineStr">
+        <is>
+          <t>0x175</t>
+        </is>
+      </c>
+      <c r="B6" s="60" t="inlineStr">
+        <is>
+          <t>SWCAN</t>
+        </is>
+      </c>
+      <c r="C6" s="60" t="inlineStr">
+        <is>
+          <t>04 00 00 — стрелка вверх</t>
+        </is>
+      </c>
+      <c r="D6" s="60" t="inlineStr">
+        <is>
+          <t>Правый блок: стрелка вверх</t>
+        </is>
+      </c>
+      <c r="E6" s="60" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="61" t="inlineStr">
+        <is>
+          <t>0x175</t>
+        </is>
+      </c>
+      <c r="B7" s="61" t="inlineStr">
+        <is>
+          <t>SWCAN</t>
+        </is>
+      </c>
+      <c r="C7" s="61" t="inlineStr">
+        <is>
+          <t>05 00 00 — стрелка вниз</t>
+        </is>
+      </c>
+      <c r="D7" s="61" t="inlineStr">
+        <is>
+          <t>Правый блок: стрелка вниз</t>
+        </is>
+      </c>
+      <c r="E7" s="61" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="60" t="inlineStr">
+        <is>
+          <t>0x175</t>
+        </is>
+      </c>
+      <c r="B8" s="60" t="inlineStr">
+        <is>
+          <t>SWCAN</t>
+        </is>
+      </c>
+      <c r="C8" s="60" t="inlineStr">
+        <is>
+          <t>01 00 01 — колесико +</t>
+        </is>
+      </c>
+      <c r="D8" s="60" t="inlineStr">
+        <is>
+          <t>Правый блок: громкость +</t>
+        </is>
+      </c>
+      <c r="E8" s="60" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="61" t="inlineStr">
+        <is>
+          <t>0x175</t>
+        </is>
+      </c>
+      <c r="B9" s="61" t="inlineStr">
+        <is>
+          <t>SWCAN</t>
+        </is>
+      </c>
+      <c r="C9" s="61" t="inlineStr">
+        <is>
+          <t>02 00 1F — колесико -</t>
+        </is>
+      </c>
+      <c r="D9" s="61" t="inlineStr">
+        <is>
+          <t>Правый блок: громкость -</t>
+        </is>
+      </c>
+      <c r="E9" s="61" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="60" t="inlineStr">
+        <is>
+          <t>0x175</t>
+        </is>
+      </c>
+      <c r="B10" s="60" t="inlineStr">
+        <is>
+          <t>SWCAN</t>
+        </is>
+      </c>
+      <c r="C10" s="60" t="inlineStr">
+        <is>
+          <t>40 00 00 — MUTE</t>
+        </is>
+      </c>
+      <c r="D10" s="60" t="inlineStr">
+        <is>
+          <t>Левый блок: MUTE</t>
+        </is>
+      </c>
+      <c r="E10" s="60" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="61" t="inlineStr">
+        <is>
+          <t>0x175</t>
+        </is>
+      </c>
+      <c r="B11" s="61" t="inlineStr">
+        <is>
+          <t>SWCAN</t>
+        </is>
+      </c>
+      <c r="C11" s="61" t="inlineStr">
+        <is>
+          <t>50 00 00 — PHONE</t>
+        </is>
+      </c>
+      <c r="D11" s="61" t="inlineStr">
+        <is>
+          <t>Левый блок: PHONE</t>
+        </is>
+      </c>
+      <c r="E11" s="61" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="60" t="inlineStr">
+        <is>
+          <t>0x175</t>
+        </is>
+      </c>
+      <c r="B12" s="60" t="inlineStr">
+        <is>
+          <t>SWCAN</t>
+        </is>
+      </c>
+      <c r="C12" s="60" t="inlineStr">
+        <is>
+          <t>10 1F 00 — колесико вверх</t>
+        </is>
+      </c>
+      <c r="D12" s="60" t="inlineStr">
+        <is>
+          <t>Левый блок: стрелка влево</t>
+        </is>
+      </c>
+      <c r="E12" s="60" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="61" t="inlineStr">
+        <is>
+          <t>0x175</t>
+        </is>
+      </c>
+      <c r="B13" s="61" t="inlineStr">
+        <is>
+          <t>SWCAN</t>
+        </is>
+      </c>
+      <c r="C13" s="61" t="inlineStr">
+        <is>
+          <t>20 01 00 — колесико вниз</t>
+        </is>
+      </c>
+      <c r="D13" s="61" t="inlineStr">
+        <is>
+          <t>Левый блок: стрелка вправо</t>
+        </is>
+      </c>
+      <c r="E13" s="61" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="60" t="inlineStr">
+        <is>
+          <t>0x170</t>
+        </is>
+      </c>
+      <c r="B14" s="60" t="inlineStr">
+        <is>
+          <t>SWCAN</t>
+        </is>
+      </c>
+      <c r="C14" s="60" t="inlineStr">
+        <is>
+          <t>byte[0]=0x20/60/72/74/76/70/30</t>
+        </is>
+      </c>
+      <c r="D14" s="60" t="inlineStr">
+        <is>
+          <t>Замок зажигания</t>
+        </is>
+      </c>
+      <c r="E14" s="60" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="61" t="inlineStr">
+        <is>
+          <t>0x235</t>
+        </is>
+      </c>
+      <c r="B15" s="61" t="inlineStr">
+        <is>
+          <t>SWCAN</t>
+        </is>
+      </c>
+      <c r="C15" s="61" t="inlineStr">
+        <is>
+          <t>byte[1] 0x00..0xFF</t>
+        </is>
+      </c>
+      <c r="D15" s="61" t="inlineStr">
+        <is>
+          <t>Яркость подсветки</t>
+        </is>
+      </c>
+      <c r="E15" s="61" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="60" t="inlineStr">
+        <is>
+          <t>0x305</t>
+        </is>
+      </c>
+      <c r="B16" s="60" t="inlineStr">
+        <is>
+          <t>SWCAN</t>
+        </is>
+      </c>
+      <c r="C16" s="60" t="inlineStr">
+        <is>
+          <t>byte[2]=0x00/40/80</t>
+        </is>
+      </c>
+      <c r="D16" s="60" t="inlineStr">
+        <is>
+          <t>Переключатель наружного освещения</t>
+        </is>
+      </c>
+      <c r="E16" s="60" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="61" t="inlineStr">
+        <is>
+          <t>0x305</t>
+        </is>
+      </c>
+      <c r="B17" s="61" t="inlineStr">
+        <is>
+          <t>SWCAN</t>
+        </is>
+      </c>
+      <c r="C17" s="61" t="inlineStr">
+        <is>
+          <t>byte[2]=0x90 (с ближним)</t>
+        </is>
+      </c>
+      <c r="D17" s="61" t="inlineStr">
+        <is>
+          <t>Задние противотуманные</t>
+        </is>
+      </c>
+      <c r="E17" s="61" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="60" t="inlineStr">
+        <is>
+          <t>0x305</t>
+        </is>
+      </c>
+      <c r="B18" s="60" t="inlineStr">
+        <is>
+          <t>SWCAN</t>
+        </is>
+      </c>
+      <c r="C18" s="60" t="inlineStr">
+        <is>
+          <t>byte[2]=0xA0 (с ближним)</t>
+        </is>
+      </c>
+      <c r="D18" s="60" t="inlineStr">
+        <is>
+          <t>Передние противотуманные</t>
+        </is>
+      </c>
+      <c r="E18" s="60" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="61" t="inlineStr">
+        <is>
+          <t>0x4E8</t>
+        </is>
+      </c>
+      <c r="B19" s="61" t="inlineStr">
+        <is>
+          <t>MSCAN</t>
+        </is>
+      </c>
+      <c r="C19" s="61" t="inlineStr">
+        <is>
+          <t>byte[6] &amp; 0x04</t>
+        </is>
+      </c>
+      <c r="D19" s="61" t="inlineStr">
+        <is>
+          <t>Задний ход</t>
+        </is>
+      </c>
+      <c r="E19" s="61" t="inlineStr">
+        <is>
+          <t>MSCAN 95.2kbps / Corsa D 2011</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="60" t="inlineStr">
+        <is>
+          <t>0x4E8</t>
+        </is>
+      </c>
+      <c r="B20" s="60" t="inlineStr">
+        <is>
+          <t>MSCAN</t>
+        </is>
+      </c>
+      <c r="C20" s="60" t="inlineStr">
+        <is>
+          <t>byte[6] &amp; 0x01</t>
+        </is>
+      </c>
+      <c r="D20" s="60" t="inlineStr">
+        <is>
+          <t>Двигатель запущен</t>
+        </is>
+      </c>
+      <c r="E20" s="60" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="61" t="inlineStr">
+        <is>
+          <t>0x450</t>
+        </is>
+      </c>
+      <c r="B21" s="61" t="inlineStr">
+        <is>
+          <t>MSCAN</t>
+        </is>
+      </c>
+      <c r="C21" s="61" t="inlineStr">
+        <is>
+          <t>byte[3] 0x00..0xFF</t>
+        </is>
+      </c>
+      <c r="D21" s="61" t="inlineStr">
+        <is>
+          <t>Яркость подсветки (плавно)</t>
+        </is>
+      </c>
+      <c r="E21" s="61" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="60" t="inlineStr">
+        <is>
+          <t>0x450</t>
+        </is>
+      </c>
+      <c r="B22" s="60" t="inlineStr">
+        <is>
+          <t>MSCAN</t>
+        </is>
+      </c>
+      <c r="C22" s="60" t="inlineStr">
+        <is>
+          <t>byte[2]=0x00/04/05/06/07</t>
+        </is>
+      </c>
+      <c r="D22" s="60" t="inlineStr">
+        <is>
+          <t>Замок зажигания</t>
+        </is>
+      </c>
+      <c r="E22" s="60" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="61" t="inlineStr">
+        <is>
+          <t>0x206</t>
+        </is>
+      </c>
+      <c r="B23" s="61" t="inlineStr">
+        <is>
+          <t>MSCAN</t>
+        </is>
+      </c>
+      <c r="C23" s="61" t="inlineStr">
+        <is>
+          <t>byte[0:2]</t>
+        </is>
+      </c>
+      <c r="D23" s="61" t="inlineStr">
+        <is>
+          <t>Кнопки мультимедиа на руле</t>
+        </is>
+      </c>
+      <c r="E23" s="61" t="inlineStr">
+        <is>
+          <t>Только при нажатии</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -5139,7 +5734,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -5989,7 +6584,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -6104,7 +6699,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -6195,7 +6790,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="001A6B1A"/>
@@ -19550,4 +20145,3872 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E9"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="9" customWidth="1" min="1" max="1"/>
+    <col width="6" customWidth="1" min="2" max="2"/>
+    <col width="11" customWidth="1" min="3" max="3"/>
+    <col width="38" customWidth="1" min="4" max="4"/>
+    <col width="34" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="59" t="inlineStr">
+        <is>
+          <t>CAN ID</t>
+        </is>
+      </c>
+      <c r="B1" s="59" t="inlineStr">
+        <is>
+          <t>DLC</t>
+        </is>
+      </c>
+      <c r="C1" s="59" t="inlineStr">
+        <is>
+          <t>Байт/Бит</t>
+        </is>
+      </c>
+      <c r="D1" s="59" t="inlineStr">
+        <is>
+          <t>Назначение</t>
+        </is>
+      </c>
+      <c r="E1" s="59" t="inlineStr">
+        <is>
+          <t>Примечание</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="60" t="inlineStr">
+        <is>
+          <t>0x1A8</t>
+        </is>
+      </c>
+      <c r="B2" s="60" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C2" s="60" t="inlineStr">
+        <is>
+          <t>0x01</t>
+        </is>
+      </c>
+      <c r="D2" s="60" t="inlineStr">
+        <is>
+          <t>Стрелка вверх (руль, левая сторона)</t>
+        </is>
+      </c>
+      <c r="E2" s="60" t="inlineStr">
+        <is>
+          <t>CAN салонная / Mercedes 203/463</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="61" t="inlineStr">
+        <is>
+          <t>0x1A8</t>
+        </is>
+      </c>
+      <c r="B3" s="61" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C3" s="61" t="inlineStr">
+        <is>
+          <t>0x02</t>
+        </is>
+      </c>
+      <c r="D3" s="61" t="inlineStr">
+        <is>
+          <t>Стрелка вниз</t>
+        </is>
+      </c>
+      <c r="E3" s="61" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="60" t="inlineStr">
+        <is>
+          <t>0x1A8</t>
+        </is>
+      </c>
+      <c r="B4" s="60" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C4" s="60" t="inlineStr">
+        <is>
+          <t>0x04</t>
+        </is>
+      </c>
+      <c r="D4" s="60" t="inlineStr">
+        <is>
+          <t>Меню вниз</t>
+        </is>
+      </c>
+      <c r="E4" s="60" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="61" t="inlineStr">
+        <is>
+          <t>0x1A8</t>
+        </is>
+      </c>
+      <c r="B5" s="61" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C5" s="61" t="inlineStr">
+        <is>
+          <t>0x08</t>
+        </is>
+      </c>
+      <c r="D5" s="61" t="inlineStr">
+        <is>
+          <t>Меню вверх</t>
+        </is>
+      </c>
+      <c r="E5" s="61" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="60" t="inlineStr">
+        <is>
+          <t>0x1A8</t>
+        </is>
+      </c>
+      <c r="B6" s="60" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C6" s="60" t="inlineStr">
+        <is>
+          <t>0x10</t>
+        </is>
+      </c>
+      <c r="D6" s="60" t="inlineStr">
+        <is>
+          <t>Громкость +</t>
+        </is>
+      </c>
+      <c r="E6" s="60" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="61" t="inlineStr">
+        <is>
+          <t>0x1A8</t>
+        </is>
+      </c>
+      <c r="B7" s="61" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C7" s="61" t="inlineStr">
+        <is>
+          <t>0x20</t>
+        </is>
+      </c>
+      <c r="D7" s="61" t="inlineStr">
+        <is>
+          <t>Громкость -</t>
+        </is>
+      </c>
+      <c r="E7" s="61" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="60" t="inlineStr">
+        <is>
+          <t>0x1A8</t>
+        </is>
+      </c>
+      <c r="B8" s="60" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C8" s="60" t="inlineStr">
+        <is>
+          <t>0x40</t>
+        </is>
+      </c>
+      <c r="D8" s="60" t="inlineStr">
+        <is>
+          <t>Трубка (вызов) вверх</t>
+        </is>
+      </c>
+      <c r="E8" s="60" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="61" t="inlineStr">
+        <is>
+          <t>0x1A8</t>
+        </is>
+      </c>
+      <c r="B9" s="61" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="C9" s="61" t="inlineStr">
+        <is>
+          <t>0x80</t>
+        </is>
+      </c>
+      <c r="D9" s="61" t="inlineStr">
+        <is>
+          <t>Трубка (вызов) вниз</t>
+        </is>
+      </c>
+      <c r="E9" s="61" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E13"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="9" customWidth="1" min="1" max="1"/>
+    <col width="6" customWidth="1" min="2" max="2"/>
+    <col width="17" customWidth="1" min="3" max="3"/>
+    <col width="32" customWidth="1" min="4" max="4"/>
+    <col width="34" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="59" t="inlineStr">
+        <is>
+          <t>CAN ID</t>
+        </is>
+      </c>
+      <c r="B1" s="59" t="inlineStr">
+        <is>
+          <t>DLC</t>
+        </is>
+      </c>
+      <c r="C1" s="59" t="inlineStr">
+        <is>
+          <t>Байт/Бит</t>
+        </is>
+      </c>
+      <c r="D1" s="59" t="inlineStr">
+        <is>
+          <t>Назначение</t>
+        </is>
+      </c>
+      <c r="E1" s="59" t="inlineStr">
+        <is>
+          <t>Примечание</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="60" t="inlineStr">
+        <is>
+          <t>0xFB</t>
+        </is>
+      </c>
+      <c r="B2" s="60" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="C2" s="60" t="inlineStr">
+        <is>
+          <t>byte[6] = 0x7F</t>
+        </is>
+      </c>
+      <c r="D2" s="60" t="inlineStr">
+        <is>
+          <t>Шатл: нейтральное положение</t>
+        </is>
+      </c>
+      <c r="E2" s="60" t="inlineStr">
+        <is>
+          <t>CAN A, 125kbps / W204 C/CLK/GLK</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="61" t="inlineStr">
+        <is>
+          <t>0xFB</t>
+        </is>
+      </c>
+      <c r="B3" s="61" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="C3" s="61" t="inlineStr">
+        <is>
+          <t>byte[6] = 0x7E</t>
+        </is>
+      </c>
+      <c r="D3" s="61" t="inlineStr">
+        <is>
+          <t>Шатл: поворот влево (шаг -1)</t>
+        </is>
+      </c>
+      <c r="E3" s="61" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="60" t="inlineStr">
+        <is>
+          <t>0xFB</t>
+        </is>
+      </c>
+      <c r="B4" s="60" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="C4" s="60" t="inlineStr">
+        <is>
+          <t>byte[6] = 0x80</t>
+        </is>
+      </c>
+      <c r="D4" s="60" t="inlineStr">
+        <is>
+          <t>Шатл: поворот вправо (шаг +1)</t>
+        </is>
+      </c>
+      <c r="E4" s="60" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="61" t="inlineStr">
+        <is>
+          <t>0xFD</t>
+        </is>
+      </c>
+      <c r="B5" s="61" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="C5" s="61" t="inlineStr">
+        <is>
+          <t>0x02</t>
+        </is>
+      </c>
+      <c r="D5" s="61" t="inlineStr">
+        <is>
+          <t>Кнопка "Назад"</t>
+        </is>
+      </c>
+      <c r="E5" s="61" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="60" t="inlineStr">
+        <is>
+          <t>0xFD</t>
+        </is>
+      </c>
+      <c r="B6" s="60" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="C6" s="60" t="inlineStr">
+        <is>
+          <t>0x20</t>
+        </is>
+      </c>
+      <c r="D6" s="60" t="inlineStr">
+        <is>
+          <t>Кнопка "C"</t>
+        </is>
+      </c>
+      <c r="E6" s="60" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="61" t="inlineStr">
+        <is>
+          <t>0xFD</t>
+        </is>
+      </c>
+      <c r="B7" s="61" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="C7" s="61" t="inlineStr">
+        <is>
+          <t>0x40 (byte[2])</t>
+        </is>
+      </c>
+      <c r="D7" s="61" t="inlineStr">
+        <is>
+          <t>Шатл: наклон влево</t>
+        </is>
+      </c>
+      <c r="E7" s="61" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="60" t="inlineStr">
+        <is>
+          <t>0xFD</t>
+        </is>
+      </c>
+      <c r="B8" s="60" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="C8" s="60" t="inlineStr">
+        <is>
+          <t>0x04 (byte[2])</t>
+        </is>
+      </c>
+      <c r="D8" s="60" t="inlineStr">
+        <is>
+          <t>Шатл: наклон вправо</t>
+        </is>
+      </c>
+      <c r="E8" s="60" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="61" t="inlineStr">
+        <is>
+          <t>0xFD</t>
+        </is>
+      </c>
+      <c r="B9" s="61" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="C9" s="61" t="inlineStr">
+        <is>
+          <t>0x10 (byte[2])</t>
+        </is>
+      </c>
+      <c r="D9" s="61" t="inlineStr">
+        <is>
+          <t>Шатл: наклон вниз</t>
+        </is>
+      </c>
+      <c r="E9" s="61" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="60" t="inlineStr">
+        <is>
+          <t>0xFD</t>
+        </is>
+      </c>
+      <c r="B10" s="60" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="C10" s="60" t="inlineStr">
+        <is>
+          <t>0x01 (byte[2])</t>
+        </is>
+      </c>
+      <c r="D10" s="60" t="inlineStr">
+        <is>
+          <t>Шатл: наклон вверх</t>
+        </is>
+      </c>
+      <c r="E10" s="60" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="61" t="inlineStr">
+        <is>
+          <t>0xFD</t>
+        </is>
+      </c>
+      <c r="B11" s="61" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="C11" s="61" t="inlineStr">
+        <is>
+          <t>0x80 (byte[2])</t>
+        </is>
+      </c>
+      <c r="D11" s="61" t="inlineStr">
+        <is>
+          <t>Кнопка шатла (нажатие)</t>
+        </is>
+      </c>
+      <c r="E11" s="61" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="60" t="inlineStr">
+        <is>
+          <t>0x428</t>
+        </is>
+      </c>
+      <c r="B12" s="60" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="C12" s="60" t="inlineStr"/>
+      <c r="D12" s="60" t="inlineStr">
+        <is>
+          <t>CAN A, шатл мультимедиа</t>
+        </is>
+      </c>
+      <c r="E12" s="60" t="inlineStr">
+        <is>
+          <t>Не расшифрован</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="61" t="inlineStr">
+        <is>
+          <t>0x747</t>
+        </is>
+      </c>
+      <c r="B13" s="61" t="inlineStr">
+        <is>
+          <t>?</t>
+        </is>
+      </c>
+      <c r="C13" s="61" t="inlineStr"/>
+      <c r="D13" s="61" t="inlineStr">
+        <is>
+          <t>CAN A, шатл мультимедиа</t>
+        </is>
+      </c>
+      <c r="E13" s="61" t="inlineStr">
+        <is>
+          <t>Не расшифрован</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="9" customWidth="1" min="1" max="1"/>
+    <col width="6" customWidth="1" min="2" max="2"/>
+    <col width="17" customWidth="1" min="3" max="3"/>
+    <col width="37" customWidth="1" min="4" max="4"/>
+    <col width="37" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="59" t="inlineStr">
+        <is>
+          <t>CAN ID</t>
+        </is>
+      </c>
+      <c r="B1" s="59" t="inlineStr">
+        <is>
+          <t>DLC</t>
+        </is>
+      </c>
+      <c r="C1" s="59" t="inlineStr">
+        <is>
+          <t>Байт/Бит</t>
+        </is>
+      </c>
+      <c r="D1" s="59" t="inlineStr">
+        <is>
+          <t>Назначение</t>
+        </is>
+      </c>
+      <c r="E1" s="59" t="inlineStr">
+        <is>
+          <t>Примечание</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="60" t="inlineStr">
+        <is>
+          <t>0x2C</t>
+        </is>
+      </c>
+      <c r="B2" s="60" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="C2" s="60" t="inlineStr">
+        <is>
+          <t>byte[1] &amp; 0x20</t>
+        </is>
+      </c>
+      <c r="D2" s="60" t="inlineStr">
+        <is>
+          <t>Аварийная сигнализация (триггер)</t>
+        </is>
+      </c>
+      <c r="E2" s="60" t="inlineStr">
+        <is>
+          <t>CAN салонная 83.3kbps / Viano W639</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="61" t="inlineStr">
+        <is>
+          <t>0x2C</t>
+        </is>
+      </c>
+      <c r="B3" s="61" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="C3" s="61" t="inlineStr">
+        <is>
+          <t>byte[3] &amp; 0x04</t>
+        </is>
+      </c>
+      <c r="D3" s="61" t="inlineStr">
+        <is>
+          <t>Левая сдвижная дверь: открыть</t>
+        </is>
+      </c>
+      <c r="E3" s="61" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="60" t="inlineStr">
+        <is>
+          <t>0x2C</t>
+        </is>
+      </c>
+      <c r="B4" s="60" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="C4" s="60" t="inlineStr">
+        <is>
+          <t>byte[3] &amp; 0x02</t>
+        </is>
+      </c>
+      <c r="D4" s="60" t="inlineStr">
+        <is>
+          <t>Левая сдвижная дверь: закрыть</t>
+        </is>
+      </c>
+      <c r="E4" s="60" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="61" t="inlineStr">
+        <is>
+          <t>0x2C</t>
+        </is>
+      </c>
+      <c r="B5" s="61" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="C5" s="61" t="inlineStr">
+        <is>
+          <t>byte[2] &amp; 0x80</t>
+        </is>
+      </c>
+      <c r="D5" s="61" t="inlineStr">
+        <is>
+          <t>Стеклоочиститель задней двери</t>
+        </is>
+      </c>
+      <c r="E5" s="61" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="60" t="inlineStr">
+        <is>
+          <t>0x2C</t>
+        </is>
+      </c>
+      <c r="B6" s="60" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="C6" s="60" t="inlineStr">
+        <is>
+          <t>byte[2] &amp; 0x40</t>
+        </is>
+      </c>
+      <c r="D6" s="60" t="inlineStr">
+        <is>
+          <t>Стеклоочиститель + омыватель задка</t>
+        </is>
+      </c>
+      <c r="E6" s="60" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="61" t="inlineStr">
+        <is>
+          <t>0x2C</t>
+        </is>
+      </c>
+      <c r="B7" s="61" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="C7" s="61" t="inlineStr">
+        <is>
+          <t>byte[3] &amp; 0x80</t>
+        </is>
+      </c>
+      <c r="D7" s="61" t="inlineStr">
+        <is>
+          <t>PTS ON/OFF</t>
+        </is>
+      </c>
+      <c r="E7" s="61" t="inlineStr">
+        <is>
+          <t>Parking Assist</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="60" t="inlineStr">
+        <is>
+          <t>0x2C</t>
+        </is>
+      </c>
+      <c r="B8" s="60" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="C8" s="60" t="inlineStr">
+        <is>
+          <t>byte[1] &amp; 0x01</t>
+        </is>
+      </c>
+      <c r="D8" s="60" t="inlineStr">
+        <is>
+          <t>ASR ON/OFF</t>
+        </is>
+      </c>
+      <c r="E8" s="60" t="inlineStr">
+        <is>
+          <t>Антипробуксовка</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="61" t="inlineStr">
+        <is>
+          <t>0x2C</t>
+        </is>
+      </c>
+      <c r="B9" s="61" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="C9" s="61" t="inlineStr">
+        <is>
+          <t>byte[2] &amp; 0x01</t>
+        </is>
+      </c>
+      <c r="D9" s="61" t="inlineStr">
+        <is>
+          <t>HZ ON/OFF</t>
+        </is>
+      </c>
+      <c r="E9" s="61" t="inlineStr">
+        <is>
+          <t>Heck...</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="60" t="inlineStr">
+        <is>
+          <t>0x2C</t>
+        </is>
+      </c>
+      <c r="B10" s="60" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="C10" s="60" t="inlineStr">
+        <is>
+          <t>byte[1] &amp; 0x10</t>
+        </is>
+      </c>
+      <c r="D10" s="60" t="inlineStr">
+        <is>
+          <t>Закрытие передних дверей</t>
+        </is>
+      </c>
+      <c r="E10" s="60" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="61" t="inlineStr">
+        <is>
+          <t>0x2C</t>
+        </is>
+      </c>
+      <c r="B11" s="61" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="C11" s="61" t="inlineStr">
+        <is>
+          <t>byte[1] &amp; 0x20</t>
+        </is>
+      </c>
+      <c r="D11" s="61" t="inlineStr">
+        <is>
+          <t>Закрытие задних дверей</t>
+        </is>
+      </c>
+      <c r="E11" s="61" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="60" t="inlineStr">
+        <is>
+          <t>0x2C</t>
+        </is>
+      </c>
+      <c r="B12" s="60" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="C12" s="60" t="inlineStr">
+        <is>
+          <t>byte[3] &amp; 0x40</t>
+        </is>
+      </c>
+      <c r="D12" s="60" t="inlineStr">
+        <is>
+          <t>Включить свет в салоне</t>
+        </is>
+      </c>
+      <c r="E12" s="60" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="61" t="inlineStr">
+        <is>
+          <t>0x2C</t>
+        </is>
+      </c>
+      <c r="B13" s="61" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="C13" s="61" t="inlineStr">
+        <is>
+          <t>byte[3] &amp; 0x80</t>
+        </is>
+      </c>
+      <c r="D13" s="61" t="inlineStr">
+        <is>
+          <t>Выключить свет в салоне</t>
+        </is>
+      </c>
+      <c r="E13" s="61" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="60" t="inlineStr">
+        <is>
+          <t>0x2C</t>
+        </is>
+      </c>
+      <c r="B14" s="60" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="C14" s="60" t="inlineStr">
+        <is>
+          <t>byte[3] &amp; 0x10</t>
+        </is>
+      </c>
+      <c r="D14" s="60" t="inlineStr">
+        <is>
+          <t>Правая сдвижная дверь: открыть</t>
+        </is>
+      </c>
+      <c r="E14" s="60" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="61" t="inlineStr">
+        <is>
+          <t>0x2C</t>
+        </is>
+      </c>
+      <c r="B15" s="61" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="C15" s="61" t="inlineStr">
+        <is>
+          <t>byte[3] &amp; 0x20</t>
+        </is>
+      </c>
+      <c r="D15" s="61" t="inlineStr">
+        <is>
+          <t>Правая сдвижная дверь: закрыть</t>
+        </is>
+      </c>
+      <c r="E15" s="61" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E14"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="9" customWidth="1" min="1" max="1"/>
+    <col width="6" customWidth="1" min="2" max="2"/>
+    <col width="21" customWidth="1" min="3" max="3"/>
+    <col width="48" customWidth="1" min="4" max="4"/>
+    <col width="24" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="59" t="inlineStr">
+        <is>
+          <t>CAN ID</t>
+        </is>
+      </c>
+      <c r="B1" s="59" t="inlineStr">
+        <is>
+          <t>DLC</t>
+        </is>
+      </c>
+      <c r="C1" s="59" t="inlineStr">
+        <is>
+          <t>Байт/Бит</t>
+        </is>
+      </c>
+      <c r="D1" s="59" t="inlineStr">
+        <is>
+          <t>Назначение</t>
+        </is>
+      </c>
+      <c r="E1" s="59" t="inlineStr">
+        <is>
+          <t>Примечание</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="60" t="inlineStr">
+        <is>
+          <t>0x1F3</t>
+        </is>
+      </c>
+      <c r="B2" s="60" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="C2" s="60" t="inlineStr">
+        <is>
+          <t>byte[2]=0x10</t>
+        </is>
+      </c>
+      <c r="D2" s="60" t="inlineStr">
+        <is>
+          <t>Левое заднее сиденье: спинка вперед</t>
+        </is>
+      </c>
+      <c r="E2" s="60" t="inlineStr">
+        <is>
+          <t>CAN 125kbps / S W221</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="61" t="inlineStr">
+        <is>
+          <t>0x1F3</t>
+        </is>
+      </c>
+      <c r="B3" s="61" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="C3" s="61" t="inlineStr">
+        <is>
+          <t>byte[2]=0x20</t>
+        </is>
+      </c>
+      <c r="D3" s="61" t="inlineStr">
+        <is>
+          <t>Спинка назад</t>
+        </is>
+      </c>
+      <c r="E3" s="61" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="60" t="inlineStr">
+        <is>
+          <t>0x1F3</t>
+        </is>
+      </c>
+      <c r="B4" s="60" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="C4" s="60" t="inlineStr">
+        <is>
+          <t>byte[1]=0x81</t>
+        </is>
+      </c>
+      <c r="D4" s="60" t="inlineStr">
+        <is>
+          <t>Подушка сиденья вперед</t>
+        </is>
+      </c>
+      <c r="E4" s="60" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="61" t="inlineStr">
+        <is>
+          <t>0x1F3</t>
+        </is>
+      </c>
+      <c r="B5" s="61" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="C5" s="61" t="inlineStr">
+        <is>
+          <t>byte[1]=0x82</t>
+        </is>
+      </c>
+      <c r="D5" s="61" t="inlineStr">
+        <is>
+          <t>Подушка сиденья назад</t>
+        </is>
+      </c>
+      <c r="E5" s="61" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="60" t="inlineStr">
+        <is>
+          <t>0x1F3</t>
+        </is>
+      </c>
+      <c r="B6" s="60" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="C6" s="60" t="inlineStr">
+        <is>
+          <t>byte[2]=0x02</t>
+        </is>
+      </c>
+      <c r="D6" s="60" t="inlineStr">
+        <is>
+          <t>Подушка сиденья вниз</t>
+        </is>
+      </c>
+      <c r="E6" s="60" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="61" t="inlineStr">
+        <is>
+          <t>0x1F3</t>
+        </is>
+      </c>
+      <c r="B7" s="61" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="C7" s="61" t="inlineStr">
+        <is>
+          <t>byte[2]=0x01</t>
+        </is>
+      </c>
+      <c r="D7" s="61" t="inlineStr">
+        <is>
+          <t>Подушка сиденья вверх</t>
+        </is>
+      </c>
+      <c r="E7" s="61" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="60" t="inlineStr">
+        <is>
+          <t>0x1F3</t>
+        </is>
+      </c>
+      <c r="B8" s="60" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="C8" s="60" t="inlineStr">
+        <is>
+          <t>byte[3]=0x01</t>
+        </is>
+      </c>
+      <c r="D8" s="60" t="inlineStr">
+        <is>
+          <t>Вентиляция левого сиденья</t>
+        </is>
+      </c>
+      <c r="E8" s="60" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="61" t="inlineStr">
+        <is>
+          <t>0x1F3</t>
+        </is>
+      </c>
+      <c r="B9" s="61" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="C9" s="61" t="inlineStr">
+        <is>
+          <t>byte[3]=0x02</t>
+        </is>
+      </c>
+      <c r="D9" s="61" t="inlineStr">
+        <is>
+          <t>Подогрев левого сиденья</t>
+        </is>
+      </c>
+      <c r="E9" s="61" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="60" t="inlineStr">
+        <is>
+          <t>0x1F4</t>
+        </is>
+      </c>
+      <c r="B10" s="60" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="C10" s="60" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D10" s="60" t="inlineStr">
+        <is>
+          <t>Правое заднее сиденье: команды те же</t>
+        </is>
+      </c>
+      <c r="E10" s="60" t="inlineStr">
+        <is>
+          <t>ID отличный от левого</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="61" t="inlineStr">
+        <is>
+          <t>0x3BD</t>
+        </is>
+      </c>
+      <c r="B11" s="61" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="C11" s="61" t="inlineStr">
+        <is>
+          <t>byte[0]=0x03/02/01</t>
+        </is>
+      </c>
+      <c r="D11" s="61" t="inlineStr">
+        <is>
+          <t>Состояние вентиляции: 3/2/1 скорость (левое)</t>
+        </is>
+      </c>
+      <c r="E11" s="61" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="60" t="inlineStr">
+        <is>
+          <t>0x3BD</t>
+        </is>
+      </c>
+      <c r="B12" s="60" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="C12" s="60" t="inlineStr">
+        <is>
+          <t>byte[0]=0x0D/09/05</t>
+        </is>
+      </c>
+      <c r="D12" s="60" t="inlineStr">
+        <is>
+          <t>Состояние подогрева: 3/2/1 (левое)</t>
+        </is>
+      </c>
+      <c r="E12" s="60" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="61" t="inlineStr">
+        <is>
+          <t>0x3BD</t>
+        </is>
+      </c>
+      <c r="B13" s="61" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="C13" s="61" t="inlineStr">
+        <is>
+          <t>byte[1]=0x03/02/01</t>
+        </is>
+      </c>
+      <c r="D13" s="61" t="inlineStr">
+        <is>
+          <t>Состояние вентиляции: 3/2/1 скорость (правое)</t>
+        </is>
+      </c>
+      <c r="E13" s="61" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="60" t="inlineStr">
+        <is>
+          <t>0x3BD</t>
+        </is>
+      </c>
+      <c r="B14" s="60" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="C14" s="60" t="inlineStr">
+        <is>
+          <t>byte[1]=0x0C/08/04</t>
+        </is>
+      </c>
+      <c r="D14" s="60" t="inlineStr">
+        <is>
+          <t>Состояние подогрева: 3/2/1 (правое)</t>
+        </is>
+      </c>
+      <c r="E14" s="60" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E68"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="9" customWidth="1" min="1" max="1"/>
+    <col width="6" customWidth="1" min="2" max="2"/>
+    <col width="11" customWidth="1" min="3" max="3"/>
+    <col width="45" customWidth="1" min="4" max="4"/>
+    <col width="38" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="59" t="inlineStr">
+        <is>
+          <t>CAN ID</t>
+        </is>
+      </c>
+      <c r="B1" s="59" t="inlineStr">
+        <is>
+          <t>DLC</t>
+        </is>
+      </c>
+      <c r="C1" s="59" t="inlineStr">
+        <is>
+          <t>Байт/Бит</t>
+        </is>
+      </c>
+      <c r="D1" s="59" t="inlineStr">
+        <is>
+          <t>Назначение</t>
+        </is>
+      </c>
+      <c r="E1" s="59" t="inlineStr">
+        <is>
+          <t>Примечание</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="60" t="inlineStr">
+        <is>
+          <t>0x0A8</t>
+        </is>
+      </c>
+      <c r="B2" s="60" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="C2" s="60" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D2" s="60" t="inlineStr">
+        <is>
+          <t>Torque, Clutch and Brake status</t>
+        </is>
+      </c>
+      <c r="E2" s="60" t="inlineStr">
+        <is>
+          <t>BMW E8x/E9x/Mini, CAN 100kbit</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="61" t="inlineStr">
+        <is>
+          <t>0x0AA</t>
+        </is>
+      </c>
+      <c r="B3" s="61" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="C3" s="61" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D3" s="61" t="inlineStr">
+        <is>
+          <t>Engine RPM and throttle position</t>
+        </is>
+      </c>
+      <c r="E3" s="61" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="60" t="inlineStr">
+        <is>
+          <t>0x0C0</t>
+        </is>
+      </c>
+      <c r="B4" s="60" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="C4" s="60" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D4" s="60" t="inlineStr">
+        <is>
+          <t>ABS / Brake counter</t>
+        </is>
+      </c>
+      <c r="E4" s="60" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="61" t="inlineStr">
+        <is>
+          <t>0x0C4</t>
+        </is>
+      </c>
+      <c r="B5" s="61" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="C5" s="61" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D5" s="61" t="inlineStr">
+        <is>
+          <t>Steering Wheel position</t>
+        </is>
+      </c>
+      <c r="E5" s="61" t="inlineStr">
+        <is>
+          <t>См. 0x0C8</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="60" t="inlineStr">
+        <is>
+          <t>0x0C8</t>
+        </is>
+      </c>
+      <c r="B6" s="60" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="C6" s="60" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D6" s="60" t="inlineStr">
+        <is>
+          <t>Steering Wheel position (дубль)</t>
+        </is>
+      </c>
+      <c r="E6" s="60" t="inlineStr">
+        <is>
+          <t>Посылается 2x, часто вместе с 0x0C4</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="61" t="inlineStr">
+        <is>
+          <t>0x0CE</t>
+        </is>
+      </c>
+      <c r="B7" s="61" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="C7" s="61" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D7" s="61" t="inlineStr">
+        <is>
+          <t>Individual Wheel Speeds (4 пары)</t>
+        </is>
+      </c>
+      <c r="E7" s="61" t="inlineStr">
+        <is>
+          <t>D0+D1/D2+D3/D4+D5/D6+D7</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="60" t="inlineStr">
+        <is>
+          <t>0x0D7</t>
+        </is>
+      </c>
+      <c r="B8" s="60" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="C8" s="60" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D8" s="60" t="inlineStr">
+        <is>
+          <t>Counter (Airbag / Seatbelt)</t>
+        </is>
+      </c>
+      <c r="E8" s="60" t="inlineStr">
+        <is>
+          <t>Счетчик</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="61" t="inlineStr">
+        <is>
+          <t>0x0E2</t>
+        </is>
+      </c>
+      <c r="B9" s="61" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="C9" s="61" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D9" s="61" t="inlineStr">
+        <is>
+          <t>Passenger door status: Unlocked, Open</t>
+        </is>
+      </c>
+      <c r="E9" s="61" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="60" t="inlineStr">
+        <is>
+          <t>0x0E6</t>
+        </is>
+      </c>
+      <c r="B10" s="60" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="C10" s="60" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D10" s="60" t="inlineStr">
+        <is>
+          <t>Rear Passenger door status: Unlocked, Open</t>
+        </is>
+      </c>
+      <c r="E10" s="60" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="61" t="inlineStr">
+        <is>
+          <t>0x0EA</t>
+        </is>
+      </c>
+      <c r="B11" s="61" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="C11" s="61" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D11" s="61" t="inlineStr">
+        <is>
+          <t>Driver door status: Unlocked, Open</t>
+        </is>
+      </c>
+      <c r="E11" s="61" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="60" t="inlineStr">
+        <is>
+          <t>0x0EE</t>
+        </is>
+      </c>
+      <c r="B12" s="60" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="C12" s="60" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D12" s="60" t="inlineStr">
+        <is>
+          <t>Rear Driver door status: Unlocked, Open</t>
+        </is>
+      </c>
+      <c r="E12" s="60" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="61" t="inlineStr">
+        <is>
+          <t>0x0F2</t>
+        </is>
+      </c>
+      <c r="B13" s="61" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="C13" s="61" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D13" s="61" t="inlineStr">
+        <is>
+          <t>Boot status: Unlocked, release, Open</t>
+        </is>
+      </c>
+      <c r="E13" s="61" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="60" t="inlineStr">
+        <is>
+          <t>0x0FA</t>
+        </is>
+      </c>
+      <c r="B14" s="60" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="C14" s="60" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D14" s="60" t="inlineStr">
+        <is>
+          <t>Electric Window controls (Driver)</t>
+        </is>
+      </c>
+      <c r="E14" s="60" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="61" t="inlineStr">
+        <is>
+          <t>0x0FB</t>
+        </is>
+      </c>
+      <c r="B15" s="61" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="C15" s="61" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D15" s="61" t="inlineStr">
+        <is>
+          <t>Electric Window controls (Passenger)</t>
+        </is>
+      </c>
+      <c r="E15" s="61" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="60" t="inlineStr">
+        <is>
+          <t>0x130</t>
+        </is>
+      </c>
+      <c r="B16" s="60" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="C16" s="60" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D16" s="60" t="inlineStr">
+        <is>
+          <t>Ignition and Key status (Term 15 / R ON?)</t>
+        </is>
+      </c>
+      <c r="E16" s="60" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="61" t="inlineStr">
+        <is>
+          <t>0x193</t>
+        </is>
+      </c>
+      <c r="B17" s="61" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="C17" s="61" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D17" s="61" t="inlineStr">
+        <is>
+          <t>Timer &amp; Cruise control status</t>
+        </is>
+      </c>
+      <c r="E17" s="61" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="60" t="inlineStr">
+        <is>
+          <t>0x19E</t>
+        </is>
+      </c>
+      <c r="B18" s="60" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="C18" s="60" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D18" s="60" t="inlineStr">
+        <is>
+          <t>ABS / Braking force</t>
+        </is>
+      </c>
+      <c r="E18" s="60" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="61" t="inlineStr">
+        <is>
+          <t>0x1A6</t>
+        </is>
+      </c>
+      <c r="B19" s="61" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="C19" s="61" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D19" s="61" t="inlineStr">
+        <is>
+          <t>Speed, as used by the instrument cluster</t>
+        </is>
+      </c>
+      <c r="E19" s="61" t="inlineStr">
+        <is>
+          <t>где байт[7]:D0 — скорость</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="60" t="inlineStr">
+        <is>
+          <t>0x1B4</t>
+        </is>
+      </c>
+      <c r="B20" s="60" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="C20" s="60" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D20" s="60" t="inlineStr">
+        <is>
+          <t>Speed [MPH] + Handbrake status</t>
+        </is>
+      </c>
+      <c r="E20" s="60" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="61" t="inlineStr">
+        <is>
+          <t>0x1C2</t>
+        </is>
+      </c>
+      <c r="B21" s="61" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="C21" s="61" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D21" s="61" t="inlineStr">
+        <is>
+          <t>PDC (Reverse) / Front Sensor data</t>
+        </is>
+      </c>
+      <c r="E21" s="61" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="60" t="inlineStr">
+        <is>
+          <t>0x1D0</t>
+        </is>
+      </c>
+      <c r="B22" s="60" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="C22" s="60" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D22" s="60" t="inlineStr">
+        <is>
+          <t>Engine temp, Pressure sensor &amp; Handbrake</t>
+        </is>
+      </c>
+      <c r="E22" s="60" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="61" t="inlineStr">
+        <is>
+          <t>0x1D6</t>
+        </is>
+      </c>
+      <c r="B23" s="61" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="C23" s="61" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D23" s="61" t="inlineStr">
+        <is>
+          <t>MFL (Steering Wheel) Buttons</t>
+        </is>
+      </c>
+      <c r="E23" s="61" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="60" t="inlineStr">
+        <is>
+          <t>0x1E1</t>
+        </is>
+      </c>
+      <c r="B24" s="60" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="C24" s="60" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D24" s="60" t="inlineStr">
+        <is>
+          <t>Counter and Door Status (200ms intervals)</t>
+        </is>
+      </c>
+      <c r="E24" s="60" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="61" t="inlineStr">
+        <is>
+          <t>0x1E3</t>
+        </is>
+      </c>
+      <c r="B25" s="61" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="C25" s="61" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D25" s="61" t="inlineStr">
+        <is>
+          <t>Interior Light Switch</t>
+        </is>
+      </c>
+      <c r="E25" s="61" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="60" t="inlineStr">
+        <is>
+          <t>0x1EE</t>
+        </is>
+      </c>
+      <c r="B26" s="60" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="C26" s="60" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D26" s="60" t="inlineStr">
+        <is>
+          <t>Indicator Stalk position</t>
+        </is>
+      </c>
+      <c r="E26" s="60" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="61" t="inlineStr">
+        <is>
+          <t>0x1F6</t>
+        </is>
+      </c>
+      <c r="B27" s="61" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="C27" s="61" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D27" s="61" t="inlineStr">
+        <is>
+          <t>Indicator Status</t>
+        </is>
+      </c>
+      <c r="E27" s="61" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="60" t="inlineStr">
+        <is>
+          <t>0x202</t>
+        </is>
+      </c>
+      <c r="B28" s="60" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="C28" s="60" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D28" s="60" t="inlineStr">
+        <is>
+          <t>Lights (Dimmer Status)</t>
+        </is>
+      </c>
+      <c r="E28" s="60" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="61" t="inlineStr">
+        <is>
+          <t>0x21A</t>
+        </is>
+      </c>
+      <c r="B29" s="61" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="C29" s="61" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D29" s="61" t="inlineStr">
+        <is>
+          <t>Lighting Status</t>
+        </is>
+      </c>
+      <c r="E29" s="61" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="60" t="inlineStr">
+        <is>
+          <t>0x23A</t>
+        </is>
+      </c>
+      <c r="B30" s="60" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="C30" s="60" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D30" s="60" t="inlineStr">
+        <is>
+          <t>Remote Control Keyfob Actions</t>
+        </is>
+      </c>
+      <c r="E30" s="60" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="61" t="inlineStr">
+        <is>
+          <t>0x246</t>
+        </is>
+      </c>
+      <c r="B31" s="61" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="C31" s="61" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D31" s="61" t="inlineStr">
+        <is>
+          <t>Air Con, Demister Status</t>
+        </is>
+      </c>
+      <c r="E31" s="61" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="60" t="inlineStr">
+        <is>
+          <t>0x24A</t>
+        </is>
+      </c>
+      <c r="B32" s="60" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="C32" s="60" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D32" s="60" t="inlineStr">
+        <is>
+          <t>Reverse Status</t>
+        </is>
+      </c>
+      <c r="E32" s="60" t="inlineStr"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="61" t="inlineStr">
+        <is>
+          <t>0x24B</t>
+        </is>
+      </c>
+      <c r="B33" s="61" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="C33" s="61" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D33" s="61" t="inlineStr">
+        <is>
+          <t>Door status (similar to 2FC)</t>
+        </is>
+      </c>
+      <c r="E33" s="61" t="inlineStr"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="60" t="inlineStr">
+        <is>
+          <t>0x252</t>
+        </is>
+      </c>
+      <c r="B34" s="60" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="C34" s="60" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D34" s="60" t="inlineStr">
+        <is>
+          <t>Windscreen Wiper Status</t>
+        </is>
+      </c>
+      <c r="E34" s="60" t="inlineStr"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="61" t="inlineStr">
+        <is>
+          <t>0x264</t>
+        </is>
+      </c>
+      <c r="B35" s="61" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="C35" s="61" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D35" s="61" t="inlineStr">
+        <is>
+          <t>iDrive Controller (Rotary Control)</t>
+        </is>
+      </c>
+      <c r="E35" s="61" t="inlineStr"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="60" t="inlineStr">
+        <is>
+          <t>0x267</t>
+        </is>
+      </c>
+      <c r="B36" s="60" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="C36" s="60" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D36" s="60" t="inlineStr">
+        <is>
+          <t>iDrive Controller (Direction / Buttons)</t>
+        </is>
+      </c>
+      <c r="E36" s="60" t="inlineStr"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="61" t="inlineStr">
+        <is>
+          <t>0x26E</t>
+        </is>
+      </c>
+      <c r="B37" s="61" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="C37" s="61" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D37" s="61" t="inlineStr">
+        <is>
+          <t>Ignition Status</t>
+        </is>
+      </c>
+      <c r="E37" s="61" t="inlineStr"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="60" t="inlineStr">
+        <is>
+          <t>0x273</t>
+        </is>
+      </c>
+      <c r="B38" s="60" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="C38" s="60" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D38" s="60" t="inlineStr">
+        <is>
+          <t>CCC / CIC Status</t>
+        </is>
+      </c>
+      <c r="E38" s="60" t="inlineStr"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="61" t="inlineStr">
+        <is>
+          <t>0x277</t>
+        </is>
+      </c>
+      <c r="B39" s="61" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="C39" s="61" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D39" s="61" t="inlineStr">
+        <is>
+          <t>iDrive controller reply to 0x273</t>
+        </is>
+      </c>
+      <c r="E39" s="61" t="inlineStr"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="60" t="inlineStr">
+        <is>
+          <t>0x286</t>
+        </is>
+      </c>
+      <c r="B40" s="60" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="C40" s="60" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D40" s="60" t="inlineStr">
+        <is>
+          <t>Rear View Mirror, Light sensor</t>
+        </is>
+      </c>
+      <c r="E40" s="60" t="inlineStr"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="61" t="inlineStr">
+        <is>
+          <t>0x2A6</t>
+        </is>
+      </c>
+      <c r="B41" s="61" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="C41" s="61" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D41" s="61" t="inlineStr">
+        <is>
+          <t>Windscreen Wiper Controls</t>
+        </is>
+      </c>
+      <c r="E41" s="61" t="inlineStr"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="60" t="inlineStr">
+        <is>
+          <t>0x2B4</t>
+        </is>
+      </c>
+      <c r="B42" s="60" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="C42" s="60" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D42" s="60" t="inlineStr">
+        <is>
+          <t>Door locking (Via Remote Control)</t>
+        </is>
+      </c>
+      <c r="E42" s="60" t="inlineStr"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="61" t="inlineStr">
+        <is>
+          <t>0x2B8</t>
+        </is>
+      </c>
+      <c r="B43" s="61" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="C43" s="61" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D43" s="61" t="inlineStr">
+        <is>
+          <t>Reset Average Fuel / Speed</t>
+        </is>
+      </c>
+      <c r="E43" s="61" t="inlineStr"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="60" t="inlineStr">
+        <is>
+          <t>0x2BA</t>
+        </is>
+      </c>
+      <c r="B44" s="60" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="C44" s="60" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D44" s="60" t="inlineStr">
+        <is>
+          <t>Counter (Toggle / Heartbeat)</t>
+        </is>
+      </c>
+      <c r="E44" s="60" t="inlineStr"/>
+    </row>
+    <row r="45">
+      <c r="A45" s="61" t="inlineStr">
+        <is>
+          <t>0x2CA</t>
+        </is>
+      </c>
+      <c r="B45" s="61" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="C45" s="61" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D45" s="61" t="inlineStr">
+        <is>
+          <t>Outside temperature</t>
+        </is>
+      </c>
+      <c r="E45" s="61" t="inlineStr"/>
+    </row>
+    <row r="46">
+      <c r="A46" s="60" t="inlineStr">
+        <is>
+          <t>0x2D6</t>
+        </is>
+      </c>
+      <c r="B46" s="60" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="C46" s="60" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D46" s="60" t="inlineStr">
+        <is>
+          <t>Air Conditioning Status</t>
+        </is>
+      </c>
+      <c r="E46" s="60" t="inlineStr"/>
+    </row>
+    <row r="47">
+      <c r="A47" s="61" t="inlineStr">
+        <is>
+          <t>0x2E6</t>
+        </is>
+      </c>
+      <c r="B47" s="61" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="C47" s="61" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D47" s="61" t="inlineStr">
+        <is>
+          <t>Climate control status (Fan and Temp)</t>
+        </is>
+      </c>
+      <c r="E47" s="61" t="inlineStr"/>
+    </row>
+    <row r="48">
+      <c r="A48" s="60" t="inlineStr">
+        <is>
+          <t>0x2EA</t>
+        </is>
+      </c>
+      <c r="B48" s="60" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="C48" s="60" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D48" s="60" t="inlineStr">
+        <is>
+          <t>Climate control status (Passenger)</t>
+        </is>
+      </c>
+      <c r="E48" s="60" t="inlineStr"/>
+    </row>
+    <row r="49">
+      <c r="A49" s="61" t="inlineStr">
+        <is>
+          <t>0x2F8</t>
+        </is>
+      </c>
+      <c r="B49" s="61" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="C49" s="61" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D49" s="61" t="inlineStr">
+        <is>
+          <t>Report Time and Date</t>
+        </is>
+      </c>
+      <c r="E49" s="61" t="inlineStr"/>
+    </row>
+    <row r="50">
+      <c r="A50" s="60" t="inlineStr">
+        <is>
+          <t>0x2FC</t>
+        </is>
+      </c>
+      <c r="B50" s="60" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="C50" s="60" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D50" s="60" t="inlineStr">
+        <is>
+          <t>Door Status</t>
+        </is>
+      </c>
+      <c r="E50" s="60" t="inlineStr"/>
+    </row>
+    <row r="51">
+      <c r="A51" s="61" t="inlineStr">
+        <is>
+          <t>0x328</t>
+        </is>
+      </c>
+      <c r="B51" s="61" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="C51" s="61" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D51" s="61" t="inlineStr">
+        <is>
+          <t>1 Second count from battery removal/reset</t>
+        </is>
+      </c>
+      <c r="E51" s="61" t="inlineStr"/>
+    </row>
+    <row r="52">
+      <c r="A52" s="60" t="inlineStr">
+        <is>
+          <t>0x32E</t>
+        </is>
+      </c>
+      <c r="B52" s="60" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="C52" s="60" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D52" s="60" t="inlineStr">
+        <is>
+          <t>Internal Temp, Light and solar sensors</t>
+        </is>
+      </c>
+      <c r="E52" s="60" t="inlineStr"/>
+    </row>
+    <row r="53">
+      <c r="A53" s="61" t="inlineStr">
+        <is>
+          <t>0x330</t>
+        </is>
+      </c>
+      <c r="B53" s="61" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="C53" s="61" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D53" s="61" t="inlineStr">
+        <is>
+          <t>Odometer, Av Fuel and Range</t>
+        </is>
+      </c>
+      <c r="E53" s="61" t="inlineStr"/>
+    </row>
+    <row r="54">
+      <c r="A54" s="60" t="inlineStr">
+        <is>
+          <t>0x349</t>
+        </is>
+      </c>
+      <c r="B54" s="60" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="C54" s="60" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D54" s="60" t="inlineStr">
+        <is>
+          <t>Fuel Level sensors</t>
+        </is>
+      </c>
+      <c r="E54" s="60" t="inlineStr"/>
+    </row>
+    <row r="55">
+      <c r="A55" s="61" t="inlineStr">
+        <is>
+          <t>0x34F</t>
+        </is>
+      </c>
+      <c r="B55" s="61" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="C55" s="61" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D55" s="61" t="inlineStr">
+        <is>
+          <t>Handbrake status</t>
+        </is>
+      </c>
+      <c r="E55" s="61" t="inlineStr"/>
+    </row>
+    <row r="56">
+      <c r="A56" s="60" t="inlineStr">
+        <is>
+          <t>0x362</t>
+        </is>
+      </c>
+      <c r="B56" s="60" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="C56" s="60" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D56" s="60" t="inlineStr">
+        <is>
+          <t>Average MPH &amp; Average MPG</t>
+        </is>
+      </c>
+      <c r="E56" s="60" t="inlineStr"/>
+    </row>
+    <row r="57">
+      <c r="A57" s="61" t="inlineStr">
+        <is>
+          <t>0x366</t>
+        </is>
+      </c>
+      <c r="B57" s="61" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="C57" s="61" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D57" s="61" t="inlineStr">
+        <is>
+          <t>Ext Temp &amp; Range</t>
+        </is>
+      </c>
+      <c r="E57" s="61" t="inlineStr"/>
+    </row>
+    <row r="58">
+      <c r="A58" s="60" t="inlineStr">
+        <is>
+          <t>0x380</t>
+        </is>
+      </c>
+      <c r="B58" s="60" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="C58" s="60" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D58" s="60" t="inlineStr">
+        <is>
+          <t>VIN Number</t>
+        </is>
+      </c>
+      <c r="E58" s="60" t="inlineStr">
+        <is>
+          <t>VIN в ascii байтах</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="61" t="inlineStr">
+        <is>
+          <t>0x394</t>
+        </is>
+      </c>
+      <c r="B59" s="61" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="C59" s="61" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D59" s="61" t="inlineStr">
+        <is>
+          <t>Hours / Distance since last service</t>
+        </is>
+      </c>
+      <c r="E59" s="61" t="inlineStr"/>
+    </row>
+    <row r="60">
+      <c r="A60" s="60" t="inlineStr">
+        <is>
+          <t>0x39E</t>
+        </is>
+      </c>
+      <c r="B60" s="60" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="C60" s="60" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D60" s="60" t="inlineStr">
+        <is>
+          <t>Set Time and Date</t>
+        </is>
+      </c>
+      <c r="E60" s="60" t="inlineStr"/>
+    </row>
+    <row r="61">
+      <c r="A61" s="61" t="inlineStr">
+        <is>
+          <t>0x3B0</t>
+        </is>
+      </c>
+      <c r="B61" s="61" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="C61" s="61" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D61" s="61" t="inlineStr">
+        <is>
+          <t>Reverse Status</t>
+        </is>
+      </c>
+      <c r="E61" s="61" t="inlineStr"/>
+    </row>
+    <row r="62">
+      <c r="A62" s="60" t="inlineStr">
+        <is>
+          <t>0x3B4</t>
+        </is>
+      </c>
+      <c r="B62" s="60" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="C62" s="60" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D62" s="60" t="inlineStr">
+        <is>
+          <t>Battery Voltage &amp; Charge status</t>
+        </is>
+      </c>
+      <c r="E62" s="60" t="inlineStr"/>
+    </row>
+    <row r="63">
+      <c r="A63" s="61" t="inlineStr">
+        <is>
+          <t>0x3B6</t>
+        </is>
+      </c>
+      <c r="B63" s="61" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="C63" s="61" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D63" s="61" t="inlineStr">
+        <is>
+          <t>Passenger Front Window status</t>
+        </is>
+      </c>
+      <c r="E63" s="61" t="inlineStr"/>
+    </row>
+    <row r="64">
+      <c r="A64" s="60" t="inlineStr">
+        <is>
+          <t>0x3B7</t>
+        </is>
+      </c>
+      <c r="B64" s="60" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="C64" s="60" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D64" s="60" t="inlineStr">
+        <is>
+          <t>Driver Rear Window status</t>
+        </is>
+      </c>
+      <c r="E64" s="60" t="inlineStr"/>
+    </row>
+    <row r="65">
+      <c r="A65" s="61" t="inlineStr">
+        <is>
+          <t>0x3B8</t>
+        </is>
+      </c>
+      <c r="B65" s="61" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="C65" s="61" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D65" s="61" t="inlineStr">
+        <is>
+          <t>Driver Front Window status</t>
+        </is>
+      </c>
+      <c r="E65" s="61" t="inlineStr"/>
+    </row>
+    <row r="66">
+      <c r="A66" s="60" t="inlineStr">
+        <is>
+          <t>0x3B9</t>
+        </is>
+      </c>
+      <c r="B66" s="60" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="C66" s="60" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D66" s="60" t="inlineStr">
+        <is>
+          <t>Passenger Rear Window status</t>
+        </is>
+      </c>
+      <c r="E66" s="60" t="inlineStr"/>
+    </row>
+    <row r="67">
+      <c r="A67" s="61" t="inlineStr">
+        <is>
+          <t>0x581</t>
+        </is>
+      </c>
+      <c r="B67" s="61" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="C67" s="61" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D67" s="61" t="inlineStr">
+        <is>
+          <t>Seatbelt Status</t>
+        </is>
+      </c>
+      <c r="E67" s="61" t="inlineStr"/>
+    </row>
+    <row r="68">
+      <c r="A68" s="60" t="inlineStr">
+        <is>
+          <t>0x7C3</t>
+        </is>
+      </c>
+      <c r="B68" s="60" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="C68" s="60" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D68" s="60" t="inlineStr">
+        <is>
+          <t>Keyfob (security, comfort, CBS data)</t>
+        </is>
+      </c>
+      <c r="E68" s="60" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E8"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="9" customWidth="1" min="1" max="1"/>
+    <col width="6" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="39" customWidth="1" min="4" max="4"/>
+    <col width="35" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="59" t="inlineStr">
+        <is>
+          <t>CAN ID</t>
+        </is>
+      </c>
+      <c r="B1" s="59" t="inlineStr">
+        <is>
+          <t>DLC</t>
+        </is>
+      </c>
+      <c r="C1" s="59" t="inlineStr">
+        <is>
+          <t>Байт/Бит</t>
+        </is>
+      </c>
+      <c r="D1" s="59" t="inlineStr">
+        <is>
+          <t>Назначение</t>
+        </is>
+      </c>
+      <c r="E1" s="59" t="inlineStr">
+        <is>
+          <t>Примечание</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="60" t="inlineStr">
+        <is>
+          <t>0x43E</t>
+        </is>
+      </c>
+      <c r="B2" s="60" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="C2" s="60" t="inlineStr">
+        <is>
+          <t>byte[0]</t>
+        </is>
+      </c>
+      <c r="D2" s="60" t="inlineStr">
+        <is>
+          <t>Кнопки ЦЗ штатного брелока</t>
+        </is>
+      </c>
+      <c r="E2" s="60" t="inlineStr">
+        <is>
+          <t>MS CAN 125k / Mazda 3/CX-5 2011+</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="61" t="inlineStr">
+        <is>
+          <t>0x43E</t>
+        </is>
+      </c>
+      <c r="B3" s="61" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="C3" s="61" t="inlineStr">
+        <is>
+          <t>byte[4]</t>
+        </is>
+      </c>
+      <c r="D3" s="61" t="inlineStr">
+        <is>
+          <t>Двери, капот, багажник</t>
+        </is>
+      </c>
+      <c r="E3" s="61" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="60" t="inlineStr">
+        <is>
+          <t>0x43E</t>
+        </is>
+      </c>
+      <c r="B4" s="60" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="C4" s="60" t="inlineStr">
+        <is>
+          <t>byte[6]</t>
+        </is>
+      </c>
+      <c r="D4" s="60" t="inlineStr">
+        <is>
+          <t>Педаль тормоза</t>
+        </is>
+      </c>
+      <c r="E4" s="60" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="61" t="inlineStr">
+        <is>
+          <t>0x050</t>
+        </is>
+      </c>
+      <c r="B5" s="61" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="C5" s="61" t="inlineStr">
+        <is>
+          <t>byte[0]</t>
+        </is>
+      </c>
+      <c r="D5" s="61" t="inlineStr">
+        <is>
+          <t>Положение ключа зажигания</t>
+        </is>
+      </c>
+      <c r="E5" s="61" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="60" t="inlineStr">
+        <is>
+          <t>0x09A</t>
+        </is>
+      </c>
+      <c r="B6" s="60" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="C6" s="60" t="inlineStr">
+        <is>
+          <t>byte[1:2]</t>
+        </is>
+      </c>
+      <c r="D6" s="60" t="inlineStr">
+        <is>
+          <t>Аварийная сигнализация + поворотники</t>
+        </is>
+      </c>
+      <c r="E6" s="60" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="61" t="inlineStr">
+        <is>
+          <t>0x09F</t>
+        </is>
+      </c>
+      <c r="B7" s="61" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="C7" s="61" t="inlineStr">
+        <is>
+          <t>byte[0]</t>
+        </is>
+      </c>
+      <c r="D7" s="61" t="inlineStr">
+        <is>
+          <t>Ручник</t>
+        </is>
+      </c>
+      <c r="E7" s="61" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="60" t="inlineStr">
+        <is>
+          <t>0x202</t>
+        </is>
+      </c>
+      <c r="B8" s="60" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="C8" s="60" t="inlineStr">
+        <is>
+          <t>byte[0:1]</t>
+        </is>
+      </c>
+      <c r="D8" s="60" t="inlineStr">
+        <is>
+          <t>Обороты двигателя</t>
+        </is>
+      </c>
+      <c r="E8" s="60" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E20"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="9" customWidth="1" min="1" max="1"/>
+    <col width="6" customWidth="1" min="2" max="2"/>
+    <col width="19" customWidth="1" min="3" max="3"/>
+    <col width="32" customWidth="1" min="4" max="4"/>
+    <col width="36" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="59" t="inlineStr">
+        <is>
+          <t>CAN ID</t>
+        </is>
+      </c>
+      <c r="B1" s="59" t="inlineStr">
+        <is>
+          <t>DLC</t>
+        </is>
+      </c>
+      <c r="C1" s="59" t="inlineStr">
+        <is>
+          <t>Байт/Бит</t>
+        </is>
+      </c>
+      <c r="D1" s="59" t="inlineStr">
+        <is>
+          <t>Назначение</t>
+        </is>
+      </c>
+      <c r="E1" s="59" t="inlineStr">
+        <is>
+          <t>Примечание</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="60" t="inlineStr">
+        <is>
+          <t>0x412</t>
+        </is>
+      </c>
+      <c r="B2" s="60" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="C2" s="60" t="inlineStr">
+        <is>
+          <t>byte[0]=0x08</t>
+        </is>
+      </c>
+      <c r="D2" s="60" t="inlineStr">
+        <is>
+          <t>Двери: закрыты все</t>
+        </is>
+      </c>
+      <c r="E2" s="60" t="inlineStr">
+        <is>
+          <t>CAN IS 500kbps / Peugeot 508 2012</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="61" t="inlineStr">
+        <is>
+          <t>0x412</t>
+        </is>
+      </c>
+      <c r="B3" s="61" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="C3" s="61" t="inlineStr">
+        <is>
+          <t>byte[6]=0x48</t>
+        </is>
+      </c>
+      <c r="D3" s="61" t="inlineStr">
+        <is>
+          <t>Левая передняя дверь открыта</t>
+        </is>
+      </c>
+      <c r="E3" s="61" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="60" t="inlineStr">
+        <is>
+          <t>0x412</t>
+        </is>
+      </c>
+      <c r="B4" s="60" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="C4" s="60" t="inlineStr">
+        <is>
+          <t>byte[6]=0x60</t>
+        </is>
+      </c>
+      <c r="D4" s="60" t="inlineStr">
+        <is>
+          <t>Левая задняя дверь открыта</t>
+        </is>
+      </c>
+      <c r="E4" s="60" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="61" t="inlineStr">
+        <is>
+          <t>0x412</t>
+        </is>
+      </c>
+      <c r="B5" s="61" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="C5" s="61" t="inlineStr">
+        <is>
+          <t>byte[6]=0x10</t>
+        </is>
+      </c>
+      <c r="D5" s="61" t="inlineStr">
+        <is>
+          <t>Правая передняя дверь открыта</t>
+        </is>
+      </c>
+      <c r="E5" s="61" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="60" t="inlineStr">
+        <is>
+          <t>0x412</t>
+        </is>
+      </c>
+      <c r="B6" s="60" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="C6" s="60" t="inlineStr">
+        <is>
+          <t>byte[6]=0x40</t>
+        </is>
+      </c>
+      <c r="D6" s="60" t="inlineStr">
+        <is>
+          <t>Правая задняя дверь открыта</t>
+        </is>
+      </c>
+      <c r="E6" s="60" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="61" t="inlineStr">
+        <is>
+          <t>0x412</t>
+        </is>
+      </c>
+      <c r="B7" s="61" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="C7" s="61" t="inlineStr">
+        <is>
+          <t>byte[0]=0x28</t>
+        </is>
+      </c>
+      <c r="D7" s="61" t="inlineStr">
+        <is>
+          <t>Тормоз нажат (+ручник)</t>
+        </is>
+      </c>
+      <c r="E7" s="61" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="60" t="inlineStr">
+        <is>
+          <t>0x412</t>
+        </is>
+      </c>
+      <c r="B8" s="60" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="C8" s="60" t="inlineStr">
+        <is>
+          <t>byte[0]=0x00</t>
+        </is>
+      </c>
+      <c r="D8" s="60" t="inlineStr">
+        <is>
+          <t>Ручник отпущен</t>
+        </is>
+      </c>
+      <c r="E8" s="60" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="61" t="inlineStr">
+        <is>
+          <t>0x412</t>
+        </is>
+      </c>
+      <c r="B9" s="61" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="C9" s="61" t="inlineStr">
+        <is>
+          <t>byte[5]=0x57</t>
+        </is>
+      </c>
+      <c r="D9" s="61" t="inlineStr">
+        <is>
+          <t>ДВС запущен</t>
+        </is>
+      </c>
+      <c r="E9" s="61" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="60" t="inlineStr">
+        <is>
+          <t>0x412</t>
+        </is>
+      </c>
+      <c r="B10" s="60" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="C10" s="60" t="inlineStr">
+        <is>
+          <t>byte[5]=0x3C</t>
+        </is>
+      </c>
+      <c r="D10" s="60" t="inlineStr">
+        <is>
+          <t>ДВС заглушен</t>
+        </is>
+      </c>
+      <c r="E10" s="60" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="61" t="inlineStr">
+        <is>
+          <t>0x468</t>
+        </is>
+      </c>
+      <c r="B11" s="61" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="C11" s="61" t="inlineStr"/>
+      <c r="D11" s="61" t="inlineStr">
+        <is>
+          <t>АКПП: положение селектора</t>
+        </is>
+      </c>
+      <c r="E11" s="61" t="inlineStr">
+        <is>
+          <t>D0-D3 меняются</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="60" t="inlineStr">
+        <is>
+          <t>0x468</t>
+        </is>
+      </c>
+      <c r="B12" s="60" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="C12" s="60" t="inlineStr">
+        <is>
+          <t>D0=0x06, D1=0x04</t>
+        </is>
+      </c>
+      <c r="D12" s="60" t="inlineStr">
+        <is>
+          <t>P — заглушен</t>
+        </is>
+      </c>
+      <c r="E12" s="60" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="61" t="inlineStr">
+        <is>
+          <t>0x468</t>
+        </is>
+      </c>
+      <c r="B13" s="61" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="C13" s="61" t="inlineStr">
+        <is>
+          <t>D0=0x26, D1=0x08</t>
+        </is>
+      </c>
+      <c r="D13" s="61" t="inlineStr">
+        <is>
+          <t>P — запущен</t>
+        </is>
+      </c>
+      <c r="E13" s="61" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="60" t="inlineStr">
+        <is>
+          <t>0x468</t>
+        </is>
+      </c>
+      <c r="B14" s="60" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="C14" s="60" t="inlineStr">
+        <is>
+          <t>D0=0x26, D1=0x08</t>
+        </is>
+      </c>
+      <c r="D14" s="60" t="inlineStr">
+        <is>
+          <t>N — запущен</t>
+        </is>
+      </c>
+      <c r="E14" s="60" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="61" t="inlineStr">
+        <is>
+          <t>0x468</t>
+        </is>
+      </c>
+      <c r="B15" s="61" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="C15" s="61" t="inlineStr">
+        <is>
+          <t>D0=0x26, D1=0x09</t>
+        </is>
+      </c>
+      <c r="D15" s="61" t="inlineStr">
+        <is>
+          <t>D или R — запущен</t>
+        </is>
+      </c>
+      <c r="E15" s="61" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="60" t="inlineStr">
+        <is>
+          <t>0x489</t>
+        </is>
+      </c>
+      <c r="B16" s="60" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="C16" s="60" t="inlineStr"/>
+      <c r="D16" s="60" t="inlineStr">
+        <is>
+          <t>АКПП: состояние</t>
+        </is>
+      </c>
+      <c r="E16" s="60" t="inlineStr">
+        <is>
+          <t>D0 меняется</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="61" t="inlineStr">
+        <is>
+          <t>0x489</t>
+        </is>
+      </c>
+      <c r="B17" s="61" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="C17" s="61" t="inlineStr">
+        <is>
+          <t>D0=0xA2</t>
+        </is>
+      </c>
+      <c r="D17" s="61" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="E17" s="61" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="60" t="inlineStr">
+        <is>
+          <t>0x489</t>
+        </is>
+      </c>
+      <c r="B18" s="60" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="C18" s="60" t="inlineStr">
+        <is>
+          <t>D0=0x13</t>
+        </is>
+      </c>
+      <c r="D18" s="60" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="E18" s="60" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="61" t="inlineStr">
+        <is>
+          <t>0x489</t>
+        </is>
+      </c>
+      <c r="B19" s="61" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="C19" s="61" t="inlineStr">
+        <is>
+          <t>D0=0x91</t>
+        </is>
+      </c>
+      <c r="D19" s="61" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="E19" s="61" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="60" t="inlineStr">
+        <is>
+          <t>0x489</t>
+        </is>
+      </c>
+      <c r="B20" s="60" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="C20" s="60" t="inlineStr">
+        <is>
+          <t>D0=0x00</t>
+        </is>
+      </c>
+      <c r="D20" s="60" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="E20" s="60" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E9"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="9" customWidth="1" min="1" max="1"/>
+    <col width="6" customWidth="1" min="2" max="2"/>
+    <col width="49" customWidth="1" min="3" max="3"/>
+    <col width="51" customWidth="1" min="4" max="4"/>
+    <col width="24" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="59" t="inlineStr">
+        <is>
+          <t>CAN ID</t>
+        </is>
+      </c>
+      <c r="B1" s="59" t="inlineStr">
+        <is>
+          <t>DLC</t>
+        </is>
+      </c>
+      <c r="C1" s="59" t="inlineStr">
+        <is>
+          <t>Байт/Бит</t>
+        </is>
+      </c>
+      <c r="D1" s="59" t="inlineStr">
+        <is>
+          <t>Назначение</t>
+        </is>
+      </c>
+      <c r="E1" s="59" t="inlineStr">
+        <is>
+          <t>Примечание</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="60" t="inlineStr">
+        <is>
+          <t>0x030</t>
+        </is>
+      </c>
+      <c r="B2" s="60" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="C2" s="60" t="inlineStr">
+        <is>
+          <t>byte[5]</t>
+        </is>
+      </c>
+      <c r="D2" s="60" t="inlineStr">
+        <is>
+          <t>Управление зеркалами (водит. дверь)</t>
+        </is>
+      </c>
+      <c r="E2" s="60" t="inlineStr">
+        <is>
+          <t>MS-CAN / Ford Focus 3</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="61" t="inlineStr">
+        <is>
+          <t>0x030</t>
+        </is>
+      </c>
+      <c r="B3" s="61" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="C3" s="61" t="inlineStr">
+        <is>
+          <t>byte[5]=x9/xA/xB/xC</t>
+        </is>
+      </c>
+      <c r="D3" s="61" t="inlineStr">
+        <is>
+          <t>Направление правого зеркала: верх/низ/лево/право</t>
+        </is>
+      </c>
+      <c r="E3" s="61" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="60" t="inlineStr">
+        <is>
+          <t>0x030</t>
+        </is>
+      </c>
+      <c r="B4" s="60" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="C4" s="60" t="inlineStr">
+        <is>
+          <t>byte[6]=x1 (не нажато), =x9 (нажато)</t>
+        </is>
+      </c>
+      <c r="D4" s="60" t="inlineStr">
+        <is>
+          <t>Факт нажатия кнопки зеркал</t>
+        </is>
+      </c>
+      <c r="E4" s="60" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="61" t="inlineStr">
+        <is>
+          <t>0x2A0</t>
+        </is>
+      </c>
+      <c r="B5" s="61" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="C5" s="61" t="inlineStr">
+        <is>
+          <t>byte[4] — направление, byte[6:7] — угол</t>
+        </is>
+      </c>
+      <c r="D5" s="61" t="inlineStr">
+        <is>
+          <t>Угол поворота колес</t>
+        </is>
+      </c>
+      <c r="E5" s="61" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="60" t="inlineStr">
+        <is>
+          <t>0x2A0</t>
+        </is>
+      </c>
+      <c r="B6" s="60" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="C6" s="60" t="inlineStr">
+        <is>
+          <t>byte[4]=1x — лево, =3x — право</t>
+        </is>
+      </c>
+      <c r="D6" s="60" t="inlineStr">
+        <is>
+          <t>Направление поворота</t>
+        </is>
+      </c>
+      <c r="E6" s="60" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="61" t="inlineStr">
+        <is>
+          <t>0x2A0</t>
+        </is>
+      </c>
+      <c r="B7" s="61" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="C7" s="61" t="inlineStr">
+        <is>
+          <t>D6:D7, 0x8000 = центр</t>
+        </is>
+      </c>
+      <c r="D7" s="61" t="inlineStr">
+        <is>
+          <t>Угол в градусах (D6 — целые, D7 — сотые)</t>
+        </is>
+      </c>
+      <c r="E7" s="61" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="60" t="inlineStr">
+        <is>
+          <t>0x110</t>
+        </is>
+      </c>
+      <c r="B8" s="60" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="C8" s="60" t="inlineStr">
+        <is>
+          <t>byte[6] (старш.) byte[7] (младш.) в сотых км/ч</t>
+        </is>
+      </c>
+      <c r="D8" s="60" t="inlineStr">
+        <is>
+          <t>Скорость</t>
+        </is>
+      </c>
+      <c r="E8" s="60" t="inlineStr">
+        <is>
+          <t>Grand C-Max / Focus 3</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="61" t="inlineStr">
+        <is>
+          <t>0x110</t>
+        </is>
+      </c>
+      <c r="B9" s="61" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="C9" s="61" t="inlineStr">
+        <is>
+          <t>byte[4] (старш.) byte[5] (младш.) /2</t>
+        </is>
+      </c>
+      <c r="D9" s="61" t="inlineStr">
+        <is>
+          <t>Обороты двигателя</t>
+        </is>
+      </c>
+      <c r="E9" s="61" t="inlineStr">
+        <is>
+          <t>Делённые на 2</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
v2.2: speedo anti-flicker, 0x96=MAX dimmer, SCR_W fill fix, docs update
</commit_message>
<xml_diff>
--- a/Honda_Toyota_CAN_ID_Map.xlsx
+++ b/Honda_Toyota_CAN_ID_Map.xlsx
@@ -2346,6 +2346,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="13" t="inlineStr">
         <is>
@@ -3803,12 +3804,12 @@
       </c>
       <c r="E50" s="19" t="inlineStr">
         <is>
-          <t>SCM</t>
+          <t>SCM_FEEDBACK: BLINKERS, WIPERS, ODOMETER, DIMMER</t>
         </is>
       </c>
       <c r="F50" s="20" t="inlineStr">
         <is>
-          <t>BLINKERS, WIPERS, ODOMETER | ЧАСТОТА: 25 Hz | BYTE[0]bit5=LEFT_BLINKER, BYTE[0]bit6=RIGHT_BLINKER, BYTE[0]&amp;0x18=WIPER_MODE(0,8,16,24), BYTE[3:5]=ODOMETER(uint24, км)</t>
+          <t>BYTE[0]bit5=LEFT_BLINKER, BYTE[0]bit6=RIGHT_BLINKER, BYTE[0]&amp;0x18=WIPER_MODE, BYTE[1]=DIMMER(0x00=dim 0x01..0x15=smooth mid 0x96=MAX), BYTE[3:5]=ODOMETER(uint24, km)</t>
         </is>
       </c>
       <c r="G50" s="21" t="inlineStr"/>

</xml_diff>

<commit_message>
v2.2-patch1: AUTO FILTER mode + new CAN IDs + SCAN flicker fix
Added:
- AUTO FILTER mode (learn 30s → detect stable byte changes)
- 0x164 LIGHT_CONTROL: BYTE[0]=LOW_BEAM+CRUISE, BYTE[2]=FOG_LIGHTS
- 0x294 blinkers corrected: BYTE[0]=BLINKERS(0x00/0x20LEFT/0x40RIGHT)
- SCAN mode: no text flicker (static labels, number-only updates)
- Event list clipped before footer (AUTO FILTER)

Updated: README, описание проекта.md, HISTORY.md, Excel
</commit_message>
<xml_diff>
--- a/Honda_Toyota_CAN_ID_Map.xlsx
+++ b/Honda_Toyota_CAN_ID_Map.xlsx
@@ -2314,7 +2314,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G124"/>
+  <dimension ref="A1:G125"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -2346,7 +2346,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="13" t="inlineStr">
         <is>
@@ -2878,7 +2877,7 @@
           <t>honda/_steering_contro...</t>
         </is>
       </c>
-      <c r="G20" s="21" t="inlineStr"/>
+      <c r="G20" s="21" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="14" t="inlineStr">
@@ -3799,20 +3798,24 @@
       </c>
       <c r="D50" s="19" t="inlineStr">
         <is>
-          <t>Обратная связь SCM</t>
+          <t>Accord 8 (2008-2012)</t>
         </is>
       </c>
       <c r="E50" s="19" t="inlineStr">
         <is>
-          <t>SCM_FEEDBACK: BLINKERS, WIPERS, ODOMETER, DIMMER</t>
+          <t>SCM (Steering Control Module)</t>
         </is>
       </c>
       <c r="F50" s="20" t="inlineStr">
         <is>
-          <t>BYTE[0]bit5=LEFT_BLINKER, BYTE[0]bit6=RIGHT_BLINKER, BYTE[0]&amp;0x18=WIPER_MODE, BYTE[1]=DIMMER(0x00=dim 0x01..0x15=smooth mid 0x96=MAX), BYTE[3:5]=ODOMETER(uint24, km)</t>
-        </is>
-      </c>
-      <c r="G50" s="21" t="inlineStr"/>
+          <t>BYTE[0]=BLINKERS(0x00=off 0x20=LEFT 0x40=RIGHT), BYTE[0]&amp;0x18=WIPER_MODE, BYTE[1]=DIMMER(0x00=dim 0x01..0x15=smooth mid 0x96=MAX), BYTE[3:5]=ODOMETER(uint24, km)</t>
+        </is>
+      </c>
+      <c r="G50" s="21" t="inlineStr">
+        <is>
+          <t>Confirmed on real hardware v2.2</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="14" t="inlineStr">
@@ -5725,6 +5728,41 @@
         </is>
       </c>
       <c r="G124" s="58" t="inlineStr"/>
+    </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>0x164</t>
+        </is>
+      </c>
+      <c r="B125" t="n">
+        <v>356</v>
+      </c>
+      <c r="C125" t="inlineStr">
+        <is>
+          <t>LIGHT_CONTROL</t>
+        </is>
+      </c>
+      <c r="D125" t="inlineStr">
+        <is>
+          <t>Accord 8 (2008-2012)</t>
+        </is>
+      </c>
+      <c r="E125" t="inlineStr">
+        <is>
+          <t>MICU</t>
+        </is>
+      </c>
+      <c r="F125" t="inlineStr">
+        <is>
+          <t>BYTE[0]bit0=LOW_BEAM(1=on 0=off), bit5=CRUISE_CTRL(1=on 0=off), BYTE[2]=FOG_LIGHTS(0x00=off 0x20=on)</t>
+        </is>
+      </c>
+      <c r="G125" t="inlineStr">
+        <is>
+          <t>Confirmed on real hardware v2.2</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="2">

</xml_diff>